<commit_message>
Move homepage stats row under Homepage in issue tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TbLUcNPxRUqBBBz7fDi7SJ
</commit_message>
<xml_diff>
--- a/seo-geo/tracking/issue-tracker.xlsx
+++ b/seo-geo/tracking/issue-tracker.xlsx
@@ -883,12 +883,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Homepage</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>site-wide</t>
+          <t>/</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Links target: /listing-division-2/, /case-studies-2/, /logistics-division-2/, /marketing-division/.</t>
+          <t>Links target: /listing-division-2/, /logistics-division-2/, /case-studies-2/, /marketing-division/.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">

</xml_diff>